<commit_message>
Add agency partner (affiliate) program concept + backlog tasks
- New docs/07-agentur-partnerprogramm.md: lean affiliate model instead of
  white-label (client on platform, agency attributed via ?ref= link + signup
  field, 25% lifetime commission, off-the-shelf affiliate tool on Stripe =
  minimal dev; full white-label deferred until demanded)
- Excel backlog: +6 partner-program tasks (P1-P6), roadmap updated
  (affiliate lean = Phase 1-2, full white-label = later)
- Add scripts/build_xlsx.py (reproducible workbook), link doc 07 from README

https://claude.ai/code/session_013JDpec7ycgLb5kBriwRot4
</commit_message>
<xml_diff>
--- a/AMZVisuals_Relaunch_Backlog.xlsx
+++ b/AMZVisuals_Relaunch_Backlog.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Kontext &amp; Hinweise" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Aufgabenliste'!$A$3:$J$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Aufgabenliste'!$A$3:$J$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1631,8 +1631,272 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Partnerprogramm</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Neu</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Affiliate-Tool an Stripe anbinden</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Fertiges Affiliate-SaaS (Rewardful / Tolt / FirstPromoter) auf Stripe aufsetzen: Tracking-Links, Cookie-Attribution, Partner-Dashboards, recurring 25%-Provision &amp; automatische Auszahlungen. Near-zero Eigenentwicklung.</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>Entscheidung 13.06.</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr"/>
+      <c r="I27" s="5" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Partnerprogramm</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>Neu</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Agentur-Attribution bei Registrierung</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>?ref=CODE aus Affiliate-Link in Cookie speichern und User zuordnen; zusätzlich optionales Feld bei Signup 'Von einer Agentur empfohlen? (Name/Code)'. Beides schreibt referred_by_agency.</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>Entscheidung 13.06.</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr"/>
+      <c r="I28" s="5" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Partnerprogramm</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Neu</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Partner-Dashboard (lean)</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Read-only-Ansicht für Agenturen: geworbene Kunden, Umsatz, verdiente Provision, Auszahlungsstatus. V1 ggf. direkt aus dem Affiliate-Tool, später nativ.</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>Entscheidung 13.06.</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr"/>
+      <c r="I29" s="5" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Partnerprogramm</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Neu</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Partner-Landingpage + Bewerbung</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Seite /partners: Nutzen (25% lifetime, ohne Design), Funktionsweise, Bewerbungsformular -&gt; Affiliate-Link wird generiert.</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>Entscheidung 13.06.</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr"/>
+      <c r="I30" s="5" t="inlineStr"/>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Partnerprogramm</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>Neu</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>Niedrig</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Partner-Welcome-Kit</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>Onboarding-Material: kurzes Loom, 1-Seiten-Guide, Sales-Deck/Vorher-Nachher-Assets, fertige E-Mail-Templates zum Weiterleiten an Kunden. Kein Code.</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>Entscheidung 13.06.</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr"/>
+      <c r="I31" s="5" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Partnerprogramm</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Neu</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Agentur-managed Modus (optional)</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>Für Agenturen, die selbst im eigenen Account für Kunden bestellen: 25% als Dauerrabatt statt Provision; Kunden als Brands. Nutzt bestehende Strukturen.</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>Entscheidung 13.06.</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr"/>
+      <c r="I32" s="5" t="inlineStr"/>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J26"/>
+  <autoFilter ref="A3:J32"/>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
@@ -1647,7 +1911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1748,22 +2012,22 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>White-Label / Agentur-Lösung</t>
+          <t>Agentur-PARTNERPROGRAMM (Affiliate) – LEAN</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Existiert NICHT (neu) – von Jonas ASAP gewünscht</t>
+          <t>Neu – LEAN-Weg statt White-Label (Entscheidung 13.06.)</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Multi-Tenant (org_id von Anfang an!). Eigenes Branding (Logo/Farben/Subdomain), eigene Preise/Marge, Reseller-Dashboard, Rollen (Agentur-Admin/Mitarbeiter/Endkunde), Wholesale-Billing. Light-Stufe zuerst, Full-Stufe (Custom Domain, eigene Mail, API) danach.</t>
+          <t>Agenturen = Provisionspartner (25% lifetime). Kunde registriert sich direkt auf amzvisuals.ai, Zuordnung via Affiliate-Link (?ref=) + Signup-Feld. Fertiges Affiliate-Tool auf Stripe (Rewardful/Tolt/FirstPromoter) = minimal Dev. Beide Angebote (Self-Serve + Done-for-you) inkludiert. Details: docs/07.</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Phase 3</t>
+          <t>Phase 1–2</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
@@ -1775,25 +2039,52 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
+          <t>Full White-Label (später, nur bei Nachfrage)</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Existiert NICHT – aufgeschoben</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Eigene Subdomain + Branding, Client-Login unter Agenturmarke, Wholesale-Billing, API. Erst bauen, wenn mehrere große Agenturen es konkret brauchen. Voraussetzung org_id ab Tag 1 ist eingeplant.</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Phase 3+ (später)</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Niedrig</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
           <t>Done-for-you Flow (bestehend) marktreif machen</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Größtenteils gebaut, mit Blocker-Bugs</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Blocker B1/B2 fixen (Signup+Zahlung), Order→Backend stabil, Liefer-/Review-Schleife, Notifications/E-Mail (H5). Schnellster Weg zu erstem Umsatz.</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Phase 1 (zuerst)</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Blocker</t>
         </is>
@@ -1813,7 +2104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1890,58 +2181,70 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Multi-Tenancy</t>
+          <t>Agentur-Modell (Entscheidung 13.06.)</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>org_id/tenant_id von Tag 1 in Datenmodell, Auth &amp; Storage – auch wenn White-Label erst Phase 3. Nachrüsten ist teuer.</t>
+          <t>Affiliate-/Partnerprogramm statt White-Label: Kunde direkt auf amzvisuals.ai, Agentur per Affiliate-Link (?ref=) + Signup-Feld zugeordnet, 25% lifetime Provision auf alle Käufe. Fertiges Affiliate-Tool auf Stripe (Rewardful/Tolt/FirstPromoter) = minimal Dev. Skalierung braucht Marketing+Vertrieb (Close-Outbound an Agenturen). Details: docs/07.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>AI-Provider-Abstraktion</t>
+          <t>Multi-Tenancy</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Bild-/Video-Modelle hinter Interfaces (ImageProvider/VideoProvider) kapseln – Modelle ändern sich monatlich.</t>
+          <t>org_id/tenant_id von Tag 1 in Datenmodell, Auth &amp; Storage – auch wenn Full White-Label erst später. Nachrüsten ist teuer.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Gut – behalten</t>
+          <t>AI-Provider-Abstraktion</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>A+-Output-Qualität ('All the Quality, None of the Compromise'), Vorher-Nachher-Slider auf der Landing, Wettbewerber-ASIN + Inspiration-ASIN-Eingabe, Brand-/Produkt-Formulare.</t>
+          <t>Bild-/Video-Modelle hinter Interfaces (ImageProvider/VideoProvider) kapseln – Modelle ändern sich monatlich.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Methode/Grenzen</t>
+          <t>Gut – behalten</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Findings aus Loom-Transcript + 60 Video-Frames (1 fps, niedrige Qualität). Manche Klein-Texte unscharf; für exakte Kontrastwerte/feine Copy wären hochauflösende Screenshots besser.</t>
+          <t>A+-Output-Qualität ('All the Quality, None of the Compromise'), Vorher-Nachher-Slider auf der Landing, Wettbewerber-ASIN + Inspiration-ASIN-Eingabe, Brand-/Produkt-Formulare.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
+          <t>Methode/Grenzen</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Findings aus Loom-Transcript + 60 Video-Frames (1 fps, niedrige Qualität). Manche Klein-Texte unscharf; für exakte Kontrastwerte/feine Copy wären hochauflösende Screenshots besser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
           <t>Vollständige Doku</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Repo JonasK01/amzvisualsai, Branch claude/hopeful-gauss-41dvp7: docs/01–06 (Bestandsaufnahme, Produkt-Spec, Handoff, Go-to-Market, Walkthrough-Findings, UI-Review).</t>
         </is>

</xml_diff>

<commit_message>
Recommend Tolt as affiliate tool (auto Wise/Payoneer/PayPal payouts)
- Confirm lifetime 25% commission on actual paid amount
- Pick Tolt over Rewardful (Rewardful was CSV/PayPal-only historically);
  Tolt has automated Wise/Payoneer payouts, flat pricing, reads real Stripe
  charges so lifetime + net-of-discount is handled natively
- Update docs/07 and backlog task P1

https://claude.ai/code/session_013JDpec7ycgLb5kBriwRot4
</commit_message>
<xml_diff>
--- a/AMZVisuals_Relaunch_Backlog.xlsx
+++ b/AMZVisuals_Relaunch_Backlog.xlsx
@@ -1654,12 +1654,12 @@
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>Affiliate-Tool an Stripe anbinden</t>
+          <t>Affiliate-Tool an Stripe anbinden (Tolt)</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Fertiges Affiliate-SaaS (Rewardful / Tolt / FirstPromoter) auf Stripe aufsetzen: Tracking-Links, Cookie-Attribution, Partner-Dashboards, recurring 25%-Provision &amp; automatische Auszahlungen. Near-zero Eigenentwicklung.</t>
+          <t>Empfehlung TOLT (statt Rewardful): auto Auszahlungen via Wise/Payoneer/PayPal, flat ab 49$/Mo, keine Payout-Gebühren, ~15 Min Setup. Liest echte Stripe-Charges -&gt; lifetime 25% auf tatsächlich gezahlten Betrag automatisch. Liefert Tracking-Links, Cookie-Attribution, Partner-Dashboards, Auszahlungen.</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">

</xml_diff>